<commit_message>
Move entrega/ para modelo/ e ajusta o exemplo resolvido
entrega/ vira modelo/ (planilha e rubrica) com o README atualizado para os novos caminhos. Planilhas regeneradas com campos neutros (Equipe/Autores) e texto de turma removido do cenario 6 e do exemplo resolvido. Preserva as edicoes feitas no GitHub em README.md e BONUS.md.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cenarios/6-exemplo-agendapet/exemplo-agendapet.xlsx
+++ b/cenarios/6-exemplo-agendapet/exemplo-agendapet.xlsx
@@ -479,7 +479,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trabalho</t>
+          <t>Modelo</t>
         </is>
       </c>
       <c r="B1" s="2" t="inlineStr">
@@ -503,19 +503,19 @@
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Grupo</t>
+          <t>Equipe</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Demonstração do professor</t>
+          <t>Exemplo resolvido</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>Integrantes (nome e RM)</t>
+          <t>Autores</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Abas: DFD -&gt; STRIDE -&gt; DREAD -&gt; Top 5 -&gt; Controles. Células em creme são suas.</t>
+          <t>Abas: DFD -&gt; STRIDE -&gt; DREAD -&gt; Top 5 -&gt; Controles. Células em creme são para preencher.</t>
         </is>
       </c>
     </row>

</xml_diff>